<commit_message>
Fix search and logout locators
</commit_message>
<xml_diff>
--- a/SpreeCommerce_Automation/src/test/resources/spree_test_data.xlsx
+++ b/SpreeCommerce_Automation/src/test/resources/spree_test_data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="spree_registration" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
     <t>Pal</t>
   </si>
   <si>
-    <t>arpitpal31@gmail.com</t>
+    <t>arpitpal101@gmail.com</t>
   </si>
   <si>
     <t>Test@123</t>
@@ -1340,9 +1340,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="arpitpal31@gmail.com" tooltip="mailto:arpitpal31@gmail.com"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1376,7 +1373,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="arpitpal31@gmail.com" tooltip="mailto:arpitpal31@gmail.com"/>
+    <hyperlink ref="A2" r:id="rId1" display="arpitpal101@gmail.com" tooltip="mailto:arpitpal101@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>